<commit_message>
Move config constants to DB and seed data
Add DB tables and plumbing to persist rule/configuration data and load it at runtime. Creates project_types, rule_tree_nodes and rule_filter_chips tables and adds is_formula_var to properties; _seed_config_tables now populates these from existing constants where available. db_gateway gains JSON support, returns numeric height tokens (no trailing "MTR"), merges built-in/extended/dynamic options, and exposes getters for project types, supervision rates, rule tree, filter chips and formula vars. PropertyRegistry now loads tree/filter/formula data from the DB. Rule engine height parsing was made more tolerant (handles numeric values and None), defaults updated for per-structure earth counts, and various UI/data files and rules updated to match the new schema; two small DB-check scripts were removed.
</commit_message>
<xml_diff>
--- a/project_Estimate.xlsx
+++ b/project_Estimate.xlsx
@@ -57,7 +57,7 @@
       <color rgb="002F5597"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="5">
     <fill>
       <patternFill/>
     </fill>
@@ -69,8 +69,18 @@
         <fgColor rgb="004F81BD"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00D9E1F2"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00EBF1DE"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -78,11 +88,25 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="00AAAAAA"/>
+      </left>
+      <right style="thin">
+        <color rgb="00AAAAAA"/>
+      </right>
+      <top style="thin">
+        <color rgb="00AAAAAA"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00AAAAAA"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
@@ -96,6 +120,11 @@
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -461,7 +490,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G44"/>
+  <dimension ref="A1:G43"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="2" max="2"/>
@@ -478,7 +507,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Subject:   |  Type: NSC  |  Date: 09-04-2026</t>
+          <t>Subject:   |  Type: NSC  |  Date: 12-04-2026</t>
         </is>
       </c>
     </row>
@@ -539,16 +568,16 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>0110030241</t>
+          <t>0110030141</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>P C C POLE:9 Mtrs.Long</t>
+          <t>P C C POLE:8 Mtrs.Long</t>
         </is>
       </c>
       <c r="D6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
@@ -556,10 +585,10 @@
         </is>
       </c>
       <c r="F6" t="n">
-        <v>10198.28</v>
+        <v>5363.44</v>
       </c>
       <c r="G6" t="n">
-        <v>20396.56</v>
+        <v>16090.32</v>
       </c>
     </row>
     <row r="7">
@@ -568,16 +597,16 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>0910010241</t>
+          <t>0504110541</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Caution Board 11KV</t>
+          <t>G.I. Earth Spike 1833X20MM</t>
         </is>
       </c>
       <c r="D7" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
@@ -585,10 +614,10 @@
         </is>
       </c>
       <c r="F7" t="n">
-        <v>143.95</v>
+        <v>367.98</v>
       </c>
       <c r="G7" t="n">
-        <v>287.9</v>
+        <v>1103.94</v>
       </c>
     </row>
     <row r="8">
@@ -597,27 +626,27 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>0504110541</t>
+          <t>0503010811</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>G.I. Earth Spike 1833X20MM</t>
+          <t>G.I. Wire 5 MM (6 SWG)</t>
         </is>
       </c>
       <c r="D8" t="n">
-        <v>2</v>
+        <v>0.008999999999999999</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>NOS</t>
+          <t>MT</t>
         </is>
       </c>
       <c r="F8" t="n">
-        <v>367.98</v>
+        <v>136865.98</v>
       </c>
       <c r="G8" t="n">
-        <v>735.96</v>
+        <v>1268.75</v>
       </c>
     </row>
     <row r="9">
@@ -626,27 +655,27 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>0503010811</t>
+          <t>0504130332</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>G.I. Wire 5 MM (6 SWG)</t>
+          <t>G.I. Stay Set LT (1680X16MM) WRKG LD-5100KG</t>
         </is>
       </c>
       <c r="D9" t="n">
-        <v>0.016</v>
+        <v>3</v>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>MT</t>
+          <t>SET</t>
         </is>
       </c>
       <c r="F9" t="n">
-        <v>136865.98</v>
+        <v>462.17</v>
       </c>
       <c r="G9" t="n">
-        <v>2233</v>
+        <v>1386.51</v>
       </c>
     </row>
     <row r="10">
@@ -655,27 +684,27 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>0504130432</t>
+          <t>0503050611</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>G.I. Stay Set HT (1830X20MM) WRKG LD-7900KG</t>
+          <t>G.I. Stay Wire 7/2.5MM (12 SWG)</t>
         </is>
       </c>
       <c r="D10" t="n">
-        <v>2</v>
+        <v>0.012</v>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>SET</t>
+          <t>MT</t>
         </is>
       </c>
       <c r="F10" t="n">
-        <v>795.83</v>
+        <v>145404.64</v>
       </c>
       <c r="G10" t="n">
-        <v>1591.66</v>
+        <v>1744.86</v>
       </c>
     </row>
     <row r="11">
@@ -684,27 +713,27 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>0503050711</t>
+          <t>0508040741</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>G.I. Stay Wire 7/3.15MM (10 SWG)</t>
+          <t>Porcelain Guy Insulator LT</t>
         </is>
       </c>
       <c r="D11" t="n">
-        <v>0.012</v>
+        <v>3</v>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>MT</t>
+          <t>NOS</t>
         </is>
       </c>
       <c r="F11" t="n">
-        <v>142310.93</v>
+        <v>18.37</v>
       </c>
       <c r="G11" t="n">
-        <v>1707.73</v>
+        <v>55.11</v>
       </c>
     </row>
     <row r="12">
@@ -713,16 +742,16 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>0508040841</t>
+          <t>0504060941</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Porcelain Guy Insulator HT</t>
+          <t>LT Distribution Box 3Ph with Steel Strap &amp; Buckle ABC</t>
         </is>
       </c>
       <c r="D12" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E12" t="inlineStr">
         <is>
@@ -730,10 +759,10 @@
         </is>
       </c>
       <c r="F12" t="n">
-        <v>52.24</v>
+        <v>1632.58</v>
       </c>
       <c r="G12" t="n">
-        <v>104.48</v>
+        <v>4897.74</v>
       </c>
     </row>
     <row r="13">
@@ -742,27 +771,27 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>0101011311</t>
+          <t>0504027141</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>M.S Angle 65X65X6mm</t>
+          <t>IPC for ABC to ABC TEE Joint</t>
         </is>
       </c>
       <c r="D13" t="n">
-        <v>0.023</v>
+        <v>16</v>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>MT</t>
+          <t>NOS</t>
         </is>
       </c>
       <c r="F13" t="n">
-        <v>108667.24</v>
+        <v>149.17</v>
       </c>
       <c r="G13" t="n">
-        <v>2466.88</v>
+        <v>2386.72</v>
       </c>
     </row>
     <row r="14">
@@ -771,27 +800,27 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>0103011511</t>
+          <t>0505034141</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>M.S Flat 65X6 mm</t>
+          <t>Dead End Clamp LT ABC (3X70+1X16+1X50SQMM)</t>
         </is>
       </c>
       <c r="D14" t="n">
-        <v>0.003</v>
+        <v>3</v>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>MT</t>
+          <t>NOS</t>
         </is>
       </c>
       <c r="F14" t="n">
-        <v>117493.74</v>
+        <v>307.84</v>
       </c>
       <c r="G14" t="n">
-        <v>375.16</v>
+        <v>923.52</v>
       </c>
     </row>
     <row r="15">
@@ -800,16 +829,16 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>0508030541</t>
+          <t>0505030841</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>11 KV Polymer Composite Disc Insulator 45KN</t>
+          <t>Eye Hook for Anchor/Suspension Clamp</t>
         </is>
       </c>
       <c r="D15" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="E15" t="inlineStr">
         <is>
@@ -817,10 +846,10 @@
         </is>
       </c>
       <c r="F15" t="n">
-        <v>183.15</v>
+        <v>100.67</v>
       </c>
       <c r="G15" t="n">
-        <v>1098.9</v>
+        <v>402.68</v>
       </c>
     </row>
     <row r="16">
@@ -829,27 +858,27 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>0504010132</t>
+          <t>0505030641</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Composite Hardware Fittings for ACSR Weasel/Rabbit (30/50SQMM)</t>
+          <t>Suspension Clamp with Bracket 35SQMM Messenger</t>
         </is>
       </c>
       <c r="D16" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>SET</t>
+          <t>NOS</t>
         </is>
       </c>
       <c r="F16" t="n">
-        <v>327.83</v>
+        <v>352.89</v>
       </c>
       <c r="G16" t="n">
-        <v>1966.98</v>
+        <v>352.89</v>
       </c>
     </row>
     <row r="17">
@@ -858,16 +887,16 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>0503010711</t>
+          <t>0103011511</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>G.I. Wire 4 MM (8 SWG)</t>
+          <t>M.S Flat 65X6 mm</t>
         </is>
       </c>
       <c r="D17" t="n">
-        <v>0.004</v>
+        <v>0.005</v>
       </c>
       <c r="E17" t="inlineStr">
         <is>
@@ -875,39 +904,25 @@
         </is>
       </c>
       <c r="F17" t="n">
-        <v>137360.98</v>
+        <v>117493.74</v>
       </c>
       <c r="G17" t="n">
-        <v>565.9299999999999</v>
+        <v>562.74</v>
       </c>
     </row>
     <row r="18">
-      <c r="A18" t="n">
-        <v>13</v>
-      </c>
-      <c r="B18" t="inlineStr">
-        <is>
-          <t>0502010921</t>
-        </is>
-      </c>
+      <c r="A18" t="inlineStr"/>
+      <c r="B18" t="inlineStr"/>
       <c r="C18" t="inlineStr">
         <is>
-          <t>ACSR Conductor 50SQMM (Rabbit)</t>
-        </is>
-      </c>
-      <c r="D18" t="n">
-        <v>0.124</v>
-      </c>
-      <c r="E18" t="inlineStr">
-        <is>
-          <t>KM</t>
-        </is>
-      </c>
-      <c r="F18" t="n">
-        <v>62290.12</v>
-      </c>
+          <t>Material Base Total</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr"/>
+      <c r="E18" t="inlineStr"/>
+      <c r="F18" t="inlineStr"/>
       <c r="G18" t="n">
-        <v>7699.06</v>
+        <v>31175.77</v>
       </c>
     </row>
     <row r="19">
@@ -915,14 +930,14 @@
       <c r="B19" t="inlineStr"/>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Material Base Total</t>
+          <t>Add: Escalation @ 5% for FY 24-25</t>
         </is>
       </c>
       <c r="D19" t="inlineStr"/>
       <c r="E19" t="inlineStr"/>
       <c r="F19" t="inlineStr"/>
       <c r="G19" t="n">
-        <v>41230.19</v>
+        <v>1558.79</v>
       </c>
     </row>
     <row r="20">
@@ -930,14 +945,14 @@
       <c r="B20" t="inlineStr"/>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Add: Escalation @ 5% for FY 24-25</t>
+          <t>Add: Escalation @ 5% for FY 25-26</t>
         </is>
       </c>
       <c r="D20" t="inlineStr"/>
       <c r="E20" t="inlineStr"/>
       <c r="F20" t="inlineStr"/>
       <c r="G20" t="n">
-        <v>2061.51</v>
+        <v>1636.73</v>
       </c>
     </row>
     <row r="21">
@@ -945,14 +960,14 @@
       <c r="B21" t="inlineStr"/>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Add: Escalation @ 5% for FY 25-26</t>
+          <t>Add: Escalation @ 5% for FY 26-27</t>
         </is>
       </c>
       <c r="D21" t="inlineStr"/>
       <c r="E21" t="inlineStr"/>
       <c r="F21" t="inlineStr"/>
       <c r="G21" t="n">
-        <v>2164.58</v>
+        <v>1718.56</v>
       </c>
     </row>
     <row r="22">
@@ -960,65 +975,75 @@
       <c r="B22" t="inlineStr"/>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Add: Escalation @ 5% for FY 26-27</t>
+          <t>Add: Sundries @ 5%</t>
         </is>
       </c>
       <c r="D22" t="inlineStr"/>
       <c r="E22" t="inlineStr"/>
       <c r="F22" t="inlineStr"/>
       <c r="G22" t="n">
-        <v>2272.81</v>
+        <v>1804.49</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr"/>
       <c r="B23" t="inlineStr"/>
-      <c r="C23" t="inlineStr">
-        <is>
-          <t>Add: Sundries @ 5%</t>
+      <c r="C23" s="2" t="inlineStr">
+        <is>
+          <t>TOTAL MATERIAL COST (A)</t>
         </is>
       </c>
       <c r="D23" t="inlineStr"/>
       <c r="E23" t="inlineStr"/>
       <c r="F23" t="inlineStr"/>
-      <c r="G23" t="n">
-        <v>2386.45</v>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" t="inlineStr"/>
-      <c r="B24" t="inlineStr"/>
-      <c r="C24" s="2" t="inlineStr">
-        <is>
-          <t>TOTAL MATERIAL COST (A)</t>
-        </is>
-      </c>
-      <c r="D24" t="inlineStr"/>
-      <c r="E24" t="inlineStr"/>
-      <c r="F24" t="inlineStr"/>
-      <c r="G24" s="2" t="n">
-        <v>50115.55</v>
+      <c r="G23" s="2" t="n">
+        <v>37894.34</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="C25" s="2" t="inlineStr">
+        <is>
+          <t>B. ERECTION / LABOR</t>
+        </is>
       </c>
     </row>
     <row r="26">
-      <c r="C26" s="2" t="inlineStr">
-        <is>
-          <t>B. ERECTION / LABOR</t>
-        </is>
+      <c r="A26" t="n">
+        <v>1</v>
+      </c>
+      <c r="B26" t="inlineStr"/>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>Fixing of 1Ph Service Connection (without cable)</t>
+        </is>
+      </c>
+      <c r="D26" t="n">
+        <v>1</v>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>NOS</t>
+        </is>
+      </c>
+      <c r="F26" t="n">
+        <v>1578</v>
+      </c>
+      <c r="G26" t="n">
+        <v>1578</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="B27" t="inlineStr"/>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Erection of 9MTR PCC Pole (HT) Without Painted</t>
+          <t>Erection of 8MTR PCC Pole (LT) Without Painted</t>
         </is>
       </c>
       <c r="D27" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E27" t="inlineStr">
         <is>
@@ -1026,15 +1051,15 @@
         </is>
       </c>
       <c r="F27" t="n">
-        <v>2620</v>
+        <v>1501</v>
       </c>
       <c r="G27" t="n">
-        <v>5240</v>
+        <v>4503</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="B28" t="inlineStr"/>
       <c r="C28" t="inlineStr">
@@ -1043,7 +1068,7 @@
         </is>
       </c>
       <c r="D28" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E28" t="inlineStr">
         <is>
@@ -1054,21 +1079,21 @@
         <v>31</v>
       </c>
       <c r="G28" t="n">
-        <v>62</v>
+        <v>93</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="B29" t="inlineStr"/>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Fixing of Caution Board</t>
+          <t>Earthing Complete</t>
         </is>
       </c>
       <c r="D29" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E29" t="inlineStr">
         <is>
@@ -1076,74 +1101,74 @@
         </is>
       </c>
       <c r="F29" t="n">
-        <v>24</v>
+        <v>313</v>
       </c>
       <c r="G29" t="n">
-        <v>48</v>
+        <v>939</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="B30" t="inlineStr"/>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Earthing Complete</t>
+          <t>LT Stay Set Complete Labour</t>
         </is>
       </c>
       <c r="D30" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>NOS</t>
+          <t>SET</t>
         </is>
       </c>
       <c r="F30" t="n">
-        <v>313</v>
+        <v>555</v>
       </c>
       <c r="G30" t="n">
-        <v>626</v>
+        <v>1665</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="B31" t="inlineStr"/>
       <c r="C31" t="inlineStr">
         <is>
-          <t>H.T. Stay Set Complete Labour</t>
+          <t>Erection of Distribution Box LT ABC</t>
         </is>
       </c>
       <c r="D31" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>SET</t>
+          <t>NOS</t>
         </is>
       </c>
       <c r="F31" t="n">
-        <v>641</v>
+        <v>507</v>
       </c>
       <c r="G31" t="n">
-        <v>1282</v>
+        <v>1521</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="B32" t="inlineStr"/>
       <c r="C32" t="inlineStr">
         <is>
-          <t>Fabrication &amp; Fixing of CG Bracket Single Pole</t>
+          <t>Fixing of IPC Connector LT ABC</t>
         </is>
       </c>
       <c r="D32" t="n">
-        <v>2</v>
+        <v>16</v>
       </c>
       <c r="E32" t="inlineStr">
         <is>
@@ -1151,24 +1176,24 @@
         </is>
       </c>
       <c r="F32" t="n">
-        <v>237</v>
+        <v>75</v>
       </c>
       <c r="G32" t="n">
-        <v>474</v>
+        <v>1200</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="B33" t="inlineStr"/>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Fixing of 11KV Disc Insulator with Strain Hardware</t>
+          <t>Erection of Anchor/Dead End Clamp LT ABC</t>
         </is>
       </c>
       <c r="D33" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="E33" t="inlineStr">
         <is>
@@ -1176,24 +1201,24 @@
         </is>
       </c>
       <c r="F33" t="n">
-        <v>65</v>
+        <v>154</v>
       </c>
       <c r="G33" t="n">
-        <v>390</v>
+        <v>462</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B34" t="inlineStr"/>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Fixing Cross Lacing Wire</t>
+          <t>Erection of Suspension Clamp LT ABC</t>
         </is>
       </c>
       <c r="D34" t="n">
-        <v>20</v>
+        <v>1</v>
       </c>
       <c r="E34" t="inlineStr">
         <is>
@@ -1201,24 +1226,24 @@
         </is>
       </c>
       <c r="F34" t="n">
-        <v>15</v>
+        <v>154</v>
       </c>
       <c r="G34" t="n">
-        <v>300</v>
+        <v>154</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B35" t="inlineStr"/>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Stringing &amp; Sagging ACSR 50SQMM 3 Wire</t>
+          <t>Survey for L.T.O.H Line</t>
         </is>
       </c>
       <c r="D35" t="n">
-        <v>0.04</v>
+        <v>0.12</v>
       </c>
       <c r="E35" t="inlineStr">
         <is>
@@ -1226,57 +1251,47 @@
         </is>
       </c>
       <c r="F35" t="n">
-        <v>8289</v>
+        <v>1714</v>
       </c>
       <c r="G35" t="n">
-        <v>331.56</v>
+        <v>205.68</v>
       </c>
     </row>
     <row r="36">
-      <c r="A36" t="n">
-        <v>10</v>
-      </c>
+      <c r="A36" t="inlineStr"/>
       <c r="B36" t="inlineStr"/>
-      <c r="C36" t="inlineStr">
-        <is>
-          <t>Survey for H.T.O.H Line</t>
-        </is>
-      </c>
-      <c r="D36" t="n">
-        <v>0.04</v>
-      </c>
-      <c r="E36" t="inlineStr">
-        <is>
-          <t>KM</t>
-        </is>
-      </c>
-      <c r="F36" t="n">
-        <v>2761</v>
-      </c>
-      <c r="G36" t="n">
-        <v>110.44</v>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" t="inlineStr"/>
-      <c r="B37" t="inlineStr"/>
-      <c r="C37" s="2" t="inlineStr">
+      <c r="C36" s="2" t="inlineStr">
         <is>
           <t>TOTAL LABOR COST (B)</t>
         </is>
       </c>
-      <c r="D37" t="inlineStr"/>
-      <c r="E37" t="inlineStr"/>
-      <c r="F37" t="inlineStr"/>
-      <c r="G37" s="2" t="n">
-        <v>8864</v>
+      <c r="D36" t="inlineStr"/>
+      <c r="E36" t="inlineStr"/>
+      <c r="F36" t="inlineStr"/>
+      <c r="G36" s="2" t="n">
+        <v>12320.68</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="C38" s="2" t="inlineStr">
+        <is>
+          <t>C. OVERHEADS &amp; TAXES</t>
+        </is>
       </c>
     </row>
     <row r="39">
-      <c r="C39" s="2" t="inlineStr">
-        <is>
-          <t>C. OVERHEADS &amp; TAXES</t>
-        </is>
+      <c r="A39" t="inlineStr"/>
+      <c r="B39" t="inlineStr"/>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>Supervision @ 10% on (A+B)</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr"/>
+      <c r="E39" t="inlineStr"/>
+      <c r="F39" t="inlineStr"/>
+      <c r="G39" t="n">
+        <v>5021.5</v>
       </c>
     </row>
     <row r="40">
@@ -1284,14 +1299,14 @@
       <c r="B40" t="inlineStr"/>
       <c r="C40" t="inlineStr">
         <is>
-          <t>Supervision @ 10% on (A+B)</t>
+          <t>GST @ 18% on Labour only</t>
         </is>
       </c>
       <c r="D40" t="inlineStr"/>
       <c r="E40" t="inlineStr"/>
       <c r="F40" t="inlineStr"/>
       <c r="G40" t="n">
-        <v>5897.96</v>
+        <v>2217.72</v>
       </c>
     </row>
     <row r="41">
@@ -1299,14 +1314,14 @@
       <c r="B41" t="inlineStr"/>
       <c r="C41" t="inlineStr">
         <is>
-          <t>GST @ 18% on Labour only</t>
+          <t>Sub-Total</t>
         </is>
       </c>
       <c r="D41" t="inlineStr"/>
       <c r="E41" t="inlineStr"/>
       <c r="F41" t="inlineStr"/>
       <c r="G41" t="n">
-        <v>1595.52</v>
+        <v>57454.25</v>
       </c>
     </row>
     <row r="42">
@@ -1314,44 +1329,29 @@
       <c r="B42" t="inlineStr"/>
       <c r="C42" t="inlineStr">
         <is>
-          <t>Sub-Total</t>
+          <t>Add: Cess @ 1% on (Mat+Lab+Sup)</t>
         </is>
       </c>
       <c r="D42" t="inlineStr"/>
       <c r="E42" t="inlineStr"/>
       <c r="F42" t="inlineStr"/>
       <c r="G42" t="n">
-        <v>66473.03</v>
+        <v>552.37</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr"/>
       <c r="B43" t="inlineStr"/>
-      <c r="C43" t="inlineStr">
-        <is>
-          <t>Add: Cess @ 1% on (Mat+Lab+Sup)</t>
+      <c r="C43" s="3" t="inlineStr">
+        <is>
+          <t>GRAND TOTAL</t>
         </is>
       </c>
       <c r="D43" t="inlineStr"/>
       <c r="E43" t="inlineStr"/>
       <c r="F43" t="inlineStr"/>
-      <c r="G43" t="n">
-        <v>648.78</v>
-      </c>
-    </row>
-    <row r="44">
-      <c r="A44" t="inlineStr"/>
-      <c r="B44" t="inlineStr"/>
-      <c r="C44" s="3" t="inlineStr">
-        <is>
-          <t>GRAND TOTAL</t>
-        </is>
-      </c>
-      <c r="D44" t="inlineStr"/>
-      <c r="E44" t="inlineStr"/>
-      <c r="F44" t="inlineStr"/>
-      <c r="G44" s="4" t="n">
-        <v>67121.8</v>
+      <c r="G43" s="4" t="n">
+        <v>58006.61</v>
       </c>
     </row>
   </sheetData>
@@ -1370,7 +1370,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F2"/>
+  <dimension ref="A1:F11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -1395,6 +1395,166 @@
         </is>
       </c>
     </row>
+    <row r="3">
+      <c r="A3" s="7" t="inlineStr">
+        <is>
+          <t>E</t>
+        </is>
+      </c>
+      <c r="B3" s="7" t="inlineStr">
+        <is>
+          <t>M.S. Flat (65X6mm)</t>
+        </is>
+      </c>
+      <c r="C3" s="7" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="D3" s="7" t="inlineStr">
+        <is>
+          <t>Lgth(m)</t>
+        </is>
+      </c>
+      <c r="E3" s="7" t="inlineStr">
+        <is>
+          <t>Total(m)</t>
+        </is>
+      </c>
+      <c r="F3" s="7" t="inlineStr">
+        <is>
+          <t>Wt(kg)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="B4" s="8" t="inlineStr">
+        <is>
+          <t>AB Cable Span (Flat)</t>
+        </is>
+      </c>
+      <c r="C4" s="8" t="n">
+        <v>3</v>
+      </c>
+      <c r="D4" s="8" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="E4" s="8" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="F4" s="8" t="n">
+        <v>4.65</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="8" t="n">
+        <v>2</v>
+      </c>
+      <c r="B5" s="8" t="inlineStr">
+        <is>
+          <t>Add: Wastage + Sag @ 3%</t>
+        </is>
+      </c>
+      <c r="C5" s="8" t="inlineStr"/>
+      <c r="D5" s="8" t="inlineStr"/>
+      <c r="E5" s="8" t="n">
+        <v>0.045</v>
+      </c>
+      <c r="F5" s="8" t="n">
+        <v>0.14</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="9" t="n"/>
+      <c r="B6" s="10" t="inlineStr">
+        <is>
+          <t>Total (incl. 3% wastage &amp; sag)</t>
+        </is>
+      </c>
+      <c r="C6" s="9" t="n"/>
+      <c r="D6" s="9" t="n"/>
+      <c r="E6" s="10" t="n">
+        <v>1.545</v>
+      </c>
+      <c r="F6" s="10" t="n">
+        <v>4.79</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="7" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="B8" s="7" t="inlineStr">
+        <is>
+          <t>G.I. Wire 5 MM (6 SWG)</t>
+        </is>
+      </c>
+      <c r="C8" s="7" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="D8" s="11" t="inlineStr"/>
+      <c r="E8" s="11" t="inlineStr"/>
+      <c r="F8" s="7" t="inlineStr">
+        <is>
+          <t>Wt(kg)</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="B9" s="8" t="inlineStr">
+        <is>
+          <t>Earthing on New LT Pole (1 nos)</t>
+        </is>
+      </c>
+      <c r="C9" s="8" t="n">
+        <v>3</v>
+      </c>
+      <c r="D9" s="8" t="inlineStr"/>
+      <c r="E9" s="8" t="inlineStr"/>
+      <c r="F9" s="8" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="8" t="n">
+        <v>2</v>
+      </c>
+      <c r="B10" s="8" t="inlineStr">
+        <is>
+          <t>Add: Wastage + Sag @ 3%</t>
+        </is>
+      </c>
+      <c r="C10" s="8" t="inlineStr"/>
+      <c r="D10" s="8" t="inlineStr"/>
+      <c r="E10" s="8" t="inlineStr"/>
+      <c r="F10" s="8" t="n">
+        <v>0.27</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="9" t="n"/>
+      <c r="B11" s="10" t="inlineStr">
+        <is>
+          <t>Total (incl. 3% wastage &amp; sag)</t>
+        </is>
+      </c>
+      <c r="C11" s="9" t="n"/>
+      <c r="D11" s="9" t="n"/>
+      <c r="E11" s="9" t="inlineStr"/>
+      <c r="F11" s="10" t="n">
+        <v>9.27</v>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A2:F2"/>

</xml_diff>